<commit_message>
Record the rubric weight decision on Merge Notes
Merge Note #2 asked the instructor to confirm the weight-2 resolution to the
official file's rubric conflict — its rubric computes 45 while its own
Evaluation Method prices Capstone System at 30. Approved: weight 2, each
criterion 6, sheet total 30.

The note now records the decision and why the alternatives were rejected,
rather than leaving an open question in a document the faculty may read.
It also carries the follow-up: the workbook in the university system still
computes 45, so the faculty need telling, and the edit must be re-applied
after any re-issue.

No marks change — this is what the workbook already contained. Rubric weights
and the blueprint's 35/35/30/100 reconciliation are unchanged, and the
exporter is still deterministic.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/course/spec/Course_Specification_ITCS355_merged.xlsx
+++ b/course/spec/Course_Specification_ITCS355_merged.xlsx
@@ -1460,12 +1460,12 @@
       </c>
       <c r="C4" s="17" t="inlineStr">
         <is>
-          <t>INTERNAL CONFLICT IN THE OFFICIAL FILE. Column G (WEIGHT) is 3 for all five criteria, so SCORE = MAX LEVEL 3 x WEIGHT 3 = 9 each and the sheet totals 45. The same workbook's 'Evaluation Method' prices 'Capstone System' at 30. Set WEIGHT to 2, which makes each criterion 6 and the sheet total exactly 30.</t>
+          <t>INTERNAL CONFLICT IN THE OFFICIAL FILE. Column G (WEIGHT) is 3 for all five criteria, so SCORE = MAX LEVEL 3 x WEIGHT 3 = 9 each and the sheet totals 45. The same workbook's 'Evaluation Method' prices 'Capstone System' at 30, and the file gives no conversion between the two. WEIGHT is set to 2 here, which makes each criterion 6 and the sheet total exactly 30.</t>
         </is>
       </c>
       <c r="D4" s="17" t="inlineStr">
         <is>
-          <t>CONFIRM. The alternative is to keep weight 3 and reprice 'Capstone System' to 45, which then breaks the 100-mark total.</t>
+          <t>DECIDED — weight 2, approved by Dr. Pasd Putthapipat on 4 September 2026. The alternatives were rejected: repricing 'Capstone System' to 45 pushes the course total to 115, and marking out of 45 then scaling by 30/45 shows students two different numbers and creates fractional marks on appeal. Still to do: tell the faculty, because the file held in the university system continues to compute 45. Re-apply this edit after any re-issue.</t>
         </is>
       </c>
     </row>

</xml_diff>